<commit_message>
how-to: the deck's words checked against the desk, and the templates' too
Every bulk item needs a link (a title alone stops at No link); the Add
button counts; Claude tidies an event's or opportunity's Description and
moves the date, time and place to their fields; the practice queue shows
nothing until Claude is done, then the row as the Queue draws it; the
Exchange carries what Kate publishes. The upload templates say the same,
name ERC Event, and lose their dashes and the To review line.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/erc-upload-template.xlsx
+++ b/templates/erc-upload-template.xlsx
@@ -493,7 +493,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Example — Research-to-Practice Workshop</t>
+          <t>Example: Research-to-Practice Workshop</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -525,7 +525,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Example — Teacher Retention in Rural Texas</t>
+          <t>Example: Teacher Retention in Rural Texas</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -553,7 +553,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Example — Data Fellowship, 2027 Cohort</t>
+          <t>Example: Data Fellowship, 2027 Cohort</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -581,7 +581,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Example — State Board Updates Graduation Rules</t>
+          <t>Example: State Board Updates Graduation Rules</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr"/>
@@ -632,7 +632,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>1. Replace the gray example rows on the Items sheet with your own items — one row per item.</t>
+          <t>1. Replace the gray example rows on the Items sheet with your own items, one row per item.</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>3. Save the file and drop it into the bulk upload box on the ERC Content Desk.</t>
+          <t>3. Save the file and drop it on Add a doc or spreadsheet, on Submit content.</t>
         </is>
       </c>
     </row>
@@ -656,14 +656,14 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Only Title or Link is required — everything else can be blank.</t>
+          <t>Every item needs a link. Everything else can be blank.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Items without a Type are fine: they land in Sort under "To review".</t>
+          <t>Items without a Type are fine: Kate sets it.</t>
         </is>
       </c>
     </row>
@@ -685,33 +685,37 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr"/>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>ERC Event: no subtype</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>New Ed Policy Research — Working Paper, Peer-Reviewed, Report, ERC Research</t>
+          <t>New Ed Policy Research: Working Paper, Peer-Reviewed, Report, ERC Research</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Event — A&amp;M, Off-Campus, Webinar-Online</t>
+          <t>Event: A&amp;M, Off-Campus, Webinar-Online</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Opportunity — Funding &amp; Grants, Fellowships &amp; Programs, Call for Proposals, Other</t>
+          <t>Opportunity: Funding &amp; Grants, Fellowships &amp; Programs, Call for Proposals, Other</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Headline — National, Texas</t>
+          <t>Headline: National, Texas</t>
         </is>
       </c>
     </row>

</xml_diff>